<commit_message>
Updated the Baseline_cover_TEMPLATE to include a README tab and provided two example baseline cover datasets from Mote
</commit_message>
<xml_diff>
--- a/Data/Baseline_cover_TEMPLATE.xlsx
+++ b/Data/Baseline_cover_TEMPLATE.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp.sharepoint.com/sites/usgs-carbonate_budget_restoration_tool/Shared Documents/Carbonate Budget Tool Collaboration/Carbonate_Budget_Tool_Code/CarbonateBudgetRestorationTool/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="92" documentId="8_{04AD622C-265A-44CF-BFA2-BE05B0EF88AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A13C234-E044-4A8C-81F5-0E5894D1DDE1}"/>
+  <xr:revisionPtr revIDLastSave="161" documentId="8_{04AD622C-265A-44CF-BFA2-BE05B0EF88AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D156C810-3A22-4106-9F1F-189A3F56C56C}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="README" sheetId="3" r:id="rId1"/>
+    <sheet name="Coral Cover input" sheetId="1" r:id="rId2"/>
+    <sheet name="Taxon list" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,61 +40,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>tc={14C795AE-2DDD-4C02-BC9C-AAA5ED7CFF47}</author>
-    <author>tc={7749CEBA-8A59-4FF8-8E46-5BD7F65BC3F8}</author>
-    <author>Toth, Lauren T</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{14C795AE-2DDD-4C02-BC9C-AAA5ED7CFF47}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Repeat list of observed corals for each unique site. Can delete or leave unused values but do not edit names</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="1" shapeId="0" xr:uid="{7749CEBA-8A59-4FF8-8E46-5BD7F65BC3F8}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Not used for SoutheastFlorida region; Inshore, MidChannel, and Offshore only apply to Keys subregions and Bank, Lagoon, and ForeReef only apply to DryTortugas subregion</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="2" shapeId="0" xr:uid="{8467B459-29AC-4AC5-9CEB-3FCDAAB9C91F}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Toth, Lauren T:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-This will be displayed on the map
-</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="103">
   <si>
     <t>Acropora cervicornis</t>
   </si>
@@ -331,12 +280,6 @@
     <t>Unique_Site_ID</t>
   </si>
   <si>
-    <t>PI_Name</t>
-  </si>
-  <si>
-    <t>PI_Email</t>
-  </si>
-  <si>
     <t>Latitude</t>
   </si>
   <si>
@@ -362,13 +305,108 @@
   </si>
   <si>
     <t>Mycetophyllia lamarckiana</t>
+  </si>
+  <si>
+    <t>Coral Cover Data Input README:</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Step 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: Input the measured or estimated percent cover of each calcifying taxon (hard corals + crustose coralline algae) in the  "Coral Cover input" tab of this spreadsheet. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Species names must exactly match the names listed in "Taxon list" or you will receive an error. If you copy/paste Taxon names from another data source rather than using the dropdown Taxon list, please ensure your taxon names are an exact match to those in "Taxon list"</t>
+    </r>
+  </si>
+  <si>
+    <t>• Taxa can be repeated for each Unique_Site_ID</t>
+  </si>
+  <si>
+    <r>
+      <t>Step 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Input site metadata</t>
+    </r>
+  </si>
+  <si>
+    <t>• Allowable fields for Habitat within the LowerKeys, MiddleKeys, and UpperKeys Subregions include: Inshore, MidChannel, and Offshore. These designations are based on XXX; Please reference XXX if you are unsure how to classify the habitat of your site</t>
+  </si>
+  <si>
+    <t>• Allowable fields for Subregion include: DryTortugas, LowerKeys, MiddleKeys, UpperKeys, Biscayne, SoutheastFlorida; These designations are based on XXX; Please reference XXX if you are unsure where to classify your site</t>
+  </si>
+  <si>
+    <t>• Allowable fields for Habitat within the DryTortugas Subregion includes: Bank, Lagoon, and ForeReef. These designations are based on XXX; Please reference XXX if you are unsure how to classify the habitat of your site</t>
+  </si>
+  <si>
+    <t>• Habitat designations are not currently included for reefs in the Biscayne and SoutheastFlorida Subregions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• A Unique_Site_ID is required. Please try to be as descriptive as possible (e.g., LK_AwesomePatchReef_Site148_2026). More generic site names can be included in the optional field </t>
+  </si>
+  <si>
+    <t>• Latitude and Longitude for the site should be entered in decimal degrees</t>
+  </si>
+  <si>
+    <t>•  The area of the site, in m2, must be provided</t>
+  </si>
+  <si>
+    <t>POC_Name</t>
+  </si>
+  <si>
+    <t>POC_Email</t>
+  </si>
+  <si>
+    <t>•  Please provide a point of contact (POC) first and last name and email for the baseline site data so that we can contact you with questions, if necessary</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -390,23 +428,39 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -429,10 +483,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -451,9 +510,7 @@
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Toth, Lauren T" id="{72433B83-F5F2-463B-899C-BB276D1D49B8}" userId="S::ltoth@usgs.gov::b1001b07-71f3-469e-89f6-892694f0967f" providerId="AD"/>
-</personList>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -771,26 +828,96 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A1" dT="2026-06-10T16:26:04.28" personId="{72433B83-F5F2-463B-899C-BB276D1D49B8}" id="{14C795AE-2DDD-4C02-BC9C-AAA5ED7CFF47}">
-    <text>Repeat list of observed corals for each unique site. Can delete or leave unused values but do not edit names</text>
-  </threadedComment>
-  <threadedComment ref="D1" dT="2026-06-10T16:28:02.00" personId="{72433B83-F5F2-463B-899C-BB276D1D49B8}" id="{7749CEBA-8A59-4FF8-8E46-5BD7F65BC3F8}">
-    <text>Not used for SoutheastFlorida region; Inshore, MidChannel, and Offshore only apply to Keys subregions and Bank, Lagoon, and ForeReef only apply to DryTortugas subregion</text>
-  </threadedComment>
-</ThreadedComments>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{222656EB-D7BC-454F-B928-92A99E9A65CD}">
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="6.265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A1" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="B3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="B4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" s="3"/>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A6" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="B7" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="B8" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="B9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="B10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="B11" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="B12" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="B13" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="B14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA43B8BD-ADC3-43CF-846A-549918345397}">
-  <dimension ref="A1:K80"/>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA43B8BD-ADC3-43CF-846A-549918345397}">
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="3" width="13.73046875" customWidth="1"/>
     <col min="4" max="4" width="14.19921875" customWidth="1"/>
-    <col min="5" max="5" width="10.265625" customWidth="1"/>
-    <col min="6" max="6" width="13.59765625" customWidth="1"/>
+    <col min="5" max="5" width="13.59765625" customWidth="1"/>
+    <col min="6" max="6" width="10.265625" customWidth="1"/>
     <col min="7" max="7" width="9.46484375" customWidth="1"/>
     <col min="8" max="8" width="10.265625" customWidth="1"/>
     <col min="9" max="9" width="14.06640625" customWidth="1"/>
@@ -801,429 +928,34 @@
         <v>62</v>
       </c>
       <c r="B1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1" t="s">
+        <v>77</v>
+      </c>
+      <c r="G1" t="s">
+        <v>79</v>
+      </c>
+      <c r="H1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I1" t="s">
         <v>83</v>
       </c>
-      <c r="D1" t="s">
-        <v>84</v>
-      </c>
-      <c r="E1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F1" t="s">
-        <v>78</v>
-      </c>
-      <c r="G1" t="s">
-        <v>81</v>
-      </c>
-      <c r="H1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I1" t="s">
-        <v>85</v>
-      </c>
       <c r="J1" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="K1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A23" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A25" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A26" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A27" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A28" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A29" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A30" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A31" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A32" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A33" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A34" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A35" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A36" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A37" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A38" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A39" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A40" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A41" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A42" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A43" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A44" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A45" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A46" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A47" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A48" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A49" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A50" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A51" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A52" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A53" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A54" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A55" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A56" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A57" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A58" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A59" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A60" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A61" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A62" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A63" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A64" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A65" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A66" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A67" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A68" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A69" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A70" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A71" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A72" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A73" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A74" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A75" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A76" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A77" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A78" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A79" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A80" t="s">
-        <v>61</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1237,7 +969,429 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{101649E4-CD8D-4DAA-89FC-8D6C93B48E30}">
+          <x14:formula1>
+            <xm:f>'Taxon list'!$A$2:$A$80</xm:f>
+          </x14:formula1>
+          <xm:sqref>A2:A1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAEEECA6-441C-430E-B4E3-69F7F23BD6EB}">
+  <dimension ref="A1:A80"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A29" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A30" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A31" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A32" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A34" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A36" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A38" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A39" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A40" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A41" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A42" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A43" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A44" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A45" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A46" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A47" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A48" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A49" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A50" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A51" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A52" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A53" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A54" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A55" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A56" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A57" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A58" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A59" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A60" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A61" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A62" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A63" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A64" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A65" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A66" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A67" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A68" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A69" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A70" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A71" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A72" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A73" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A74" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A75" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A76" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A77" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A78" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A79" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A80" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1251,17 +1405,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000AA90A7536739341825FB392424435FB" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ca57789ecb406bb7a99068f68ac4c0ed">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="797e7fd4-719a-42b3-b312-968ffa9058ad" xmlns:ns3="811eef35-9bdd-441e-81aa-50455f68c6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="89dc4794f4784a0bac47690674a3da53" ns2:_="" ns3:_="">
     <xsd:import namespace="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
@@ -1456,6 +1599,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="811eef35-9bdd-441e-81aa-50455f68c6c3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D6BB395-747F-41BC-A23A-168993E4FE92}">
   <ds:schemaRefs>
@@ -1465,17 +1619,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9D3406C-31AD-4E38-96F6-B0246BC4EAE6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
-    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D5B4E66-2F53-40AB-B6DF-59838CE46951}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1494,6 +1637,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9D3406C-31AD-4E38-96F6-B0246BC4EAE6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
+    <ds:schemaRef ds:uri="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{6dd02d64-b7f3-43f7-a145-cfd68d338edf}" enabled="1" method="Standard" siteId="{0693b5ba-4b18-4d7b-9341-f32f400a5494}" removed="0"/>

</xml_diff>

<commit_message>
Added READMEs to Data Input TEMPLATES
</commit_message>
<xml_diff>
--- a/Data/Baseline_cover_TEMPLATE.xlsx
+++ b/Data/Baseline_cover_TEMPLATE.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="161" documentId="8_{04AD622C-265A-44CF-BFA2-BE05B0EF88AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D156C810-3A22-4106-9F1F-189A3F56C56C}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
@@ -507,10 +507,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>